<commit_message>
Kredebsial : Pengajuan Kredensial : Fix Anomali Upload Berkas
fix anomali saat upload berkas. hal ini berdampak pada proses validasi
yang dilakukan oleh admin. Untuk Sebelumnya mengalami kendala dimana
sistem tidak dapat menampilkan berkas dikarenakan berkas yang diupload merupakan data lama

Signed-off-by: unknown <maulanafajar751@gmail.com>
</commit_message>
<xml_diff>
--- a/public/file/pegawai/data-pegawai.xlsx
+++ b/public/file/pegawai/data-pegawai.xlsx
@@ -21439,9 +21439,11 @@
         <v>26</v>
       </c>
       <c r="O316" t="s">
-        <v>19</v>
-      </c>
-      <c r="P316"/>
+        <v>235</v>
+      </c>
+      <c r="P316" t="s">
+        <v>1711</v>
+      </c>
     </row>
     <row r="317" spans="1:16">
       <c r="A317">

</xml_diff>